<commit_message>
checkpoint: pre-hotfix baseline with full architecture upgrade
</commit_message>
<xml_diff>
--- a/backend/data/equipment_agent.xlsx
+++ b/backend/data/equipment_agent.xlsx
@@ -4518,7 +4518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U37"/>
+  <dimension ref="A1:U98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7475,6 +7475,4686 @@
       <c r="U37" t="inlineStr">
         <is>
           <t>2026-10-08T16:25:48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000095</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:55.668113+00:00</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:55Z</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:55Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000096</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:56Z</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000097</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000098</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>5</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000099</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000100</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>3</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000101</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000102</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>REQ-20261008-000103</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:58Z</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:48:58Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000104</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:52.199711+00:00</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:51Z</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:53Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000105</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:53Z</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:53Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000106</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:57Z</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000107</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>5</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:57Z</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000108</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:57Z</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000109</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:59Z</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:02:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000110</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:03:01Z</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:03:02Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000111</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>2</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:15:44.381460+00:00</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:15:18Z</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:15:48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000112</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:15:49Z</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:15:49Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000113</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:05Z</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:05Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000114</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>5</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:05Z</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:05Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000115</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:06Z</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:06Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000116</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>3</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:37Z</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:37Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000117</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>2</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:37Z</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:37Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000118</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:37Z</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:37Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000119</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:18:58Z</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:19:06Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000120</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:24.999688+00:00</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:23Z</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:25Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000121</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:26Z</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:26Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000122</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:30Z</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000123</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>5</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:30Z</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000124</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:30Z</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000125</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>3</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:32Z</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000126</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>2</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:33Z</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:33Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000127</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:33Z</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:33Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000128</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:35Z</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:09:36Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000129</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>2</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:13.637683+00:00</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:12Z</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:14Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000130</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:15Z</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:15Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000131</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>2</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:19Z</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:19Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000132</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>5</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:19Z</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:19Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000133</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:19Z</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:19Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000134</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>3</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:21Z</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:21Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000135</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>2</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:22Z</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:22Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000136</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:22Z</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:22Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000137</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:23Z</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:11:24Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000138</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:38.093530+00:00</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:36Z</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:38Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000139</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:39Z</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000140</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>2</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:44Z</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:44Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000141</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>5</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:44Z</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:44Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000142</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:45Z</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:45Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000143</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>3</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:47Z</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:47Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000144</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>2</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:47Z</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:47Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000145</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:47Z</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:47Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000146</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:49Z</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:15:50Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000147</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>2</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:25.832409+00:00</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:25Z</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:26Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000148</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:26Z</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:26Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000149</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>2</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:27Z</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:27Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000150</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>5</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:27Z</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:27Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000151</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>1</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:27Z</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:27Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000152</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>3</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:28Z</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:28Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000153</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>2</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:28Z</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:28Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000154</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:28Z</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:28Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000155</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>1</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:29Z</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:21:29Z</t>
         </is>
       </c>
     </row>
@@ -7489,7 +12169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34.109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7716,6 +12396,50 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>upgrade.test.user@company.com</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Upgrade Test User</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>newemp99@company.com</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Trần Văn Mới</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(agent): integrate Gemini router without fallback, fix inventory lookup and borrow/return UX
</commit_message>
<xml_diff>
--- a/backend/data/equipment_agent.xlsx
+++ b/backend/data/equipment_agent.xlsx
@@ -4518,7 +4518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U98"/>
+  <dimension ref="A1:U151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12155,6 +12155,4126 @@
       <c r="U98" t="inlineStr">
         <is>
           <t>2026-10-09T03:21:29Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000156</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>2</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:44.088657+00:00</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:43Z</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:44Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000157</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:45Z</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:45Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000158</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>2</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:48Z</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000159</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>5</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:48Z</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000160</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:48Z</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000161</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
+        <v>3</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:50Z</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:50Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000162</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>2</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:50Z</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:50Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000163</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>1</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:50Z</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:50Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000164</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>1</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:51Z</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:01:52Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000165</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>1</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:29:24Z</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:29:24Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000166</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>1</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000167</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Regression D4</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Test Item D4</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>1</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Kiểm tra D4</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000168</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Regression D6</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Test Item D6</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>1</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000169</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>other_user@company.com</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Other User</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Regression D7</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Test Item D7</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>1</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000170</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Regression D8 Overdue</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Test Item D8</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>1</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:57Z</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:56Z</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:31:57Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000171</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>1</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000172</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Regression D4</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Test Item D4</t>
+        </is>
+      </c>
+      <c r="G115" t="n">
+        <v>1</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>Kiểm tra D4</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000173</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Regression D6</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Test Item D6</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>1</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000174</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>other_user@company.com</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Other User</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Regression D7</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Test Item D7</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>1</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000175</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Regression D8 Overdue</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Test Item D8</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>1</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:33Z</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:33Z</t>
+        </is>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:32:33Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000176</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>2</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:09.808099+00:00</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:08Z</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000177</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>1</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:11Z</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:11Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000178</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>2</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:15Z</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:15Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000179</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>5</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:15Z</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:15Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000180</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G123" t="n">
+        <v>1</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:16Z</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:16Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000181</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>3</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:18Z</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:18Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000182</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G125" t="n">
+        <v>2</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:18Z</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:18Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000183</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:18Z</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:18Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000184</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G127" t="n">
+        <v>1</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:20Z</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:33:21Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000185</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>1</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:28Z</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:28Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000186</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Regression D4</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Test Item D4</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>1</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>Kiểm tra D4</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:30Z</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:29Z</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000187</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Regression D6</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Test Item D6</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>1</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:30Z</t>
+        </is>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000188</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>other_user@company.com</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Other User</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Regression D7</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Test Item D7</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>1</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:31Z</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:31Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000189</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Regression D8 Overdue</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Test Item D8</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>1</v>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:32Z</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:31Z</t>
+        </is>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:34:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000190</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
+        <v>1</v>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:50Z</t>
+        </is>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:50Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000191</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Regression D4</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Test Item D4</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>1</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>Kiểm tra D4</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:50Z</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000192</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Regression D6</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Test Item D6</t>
+        </is>
+      </c>
+      <c r="G135" t="n">
+        <v>1</v>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000193</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>other_user@company.com</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Other User</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Regression D7</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Test Item D7</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>1</v>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000194</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Regression D8 Overdue</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Test Item D8</t>
+        </is>
+      </c>
+      <c r="G137" t="n">
+        <v>1</v>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:39:51Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000195</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>regular.dev.user@company.com</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Dev User</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Test Project X</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G138" t="n">
+        <v>2</v>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Testing manager workflow in agent</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Standard testing priority</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:34.297651+00:00</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:33Z</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000196</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>test.manager@company.com</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Manager's Own Project</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G139" t="n">
+        <v>1</v>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Self-request test</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>Self created</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:36Z</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:36Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000197</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>vana@company.com</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Nguyen Van A</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Project Alpha</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G140" t="n">
+        <v>2</v>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Testing Alpha hardware</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Standard test run for Project Alpha</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:40Z</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:40Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000198</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>thib@company.com</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Tran Thi B</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Project Beta</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>5</v>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Beta board integration</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Crucial beta phase integration</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:40Z</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:40Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000199</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>vanc@company.com</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Le Van C</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Project Gamma</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G142" t="n">
+        <v>1</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Thermal sensor validation</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Critical safety validation</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:40Z</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:40Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000200</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>overdue@company.com</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Overdue Borrower</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Legacy Project</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G143" t="n">
+        <v>3</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2020-01-15</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Past testing</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:42Z</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:42Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000201</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>future@company.com</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Active Future Borrower</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Future Project</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>CSW-001</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Switch SPST 12V</t>
+        </is>
+      </c>
+      <c r="G144" t="n">
+        <v>2</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Long running project</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Long term</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:43Z</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:43Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000202</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>approved@company.com</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Approved Only Person</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Pending Handover Project</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>EBS-001</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Sensor Temp I2C</t>
+        </is>
+      </c>
+      <c r="G145" t="n">
+        <v>1</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Not yet handed over</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:43Z</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:43Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000203</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>manager.alpha@company.com</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Manager 1</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Alpha Project</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G146" t="n">
+        <v>1</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>M1 testing</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:45Z</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:40:45Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000204</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G147" t="n">
+        <v>1</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:14Z</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:14Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000205</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Regression D4</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Test Item D4</t>
+        </is>
+      </c>
+      <c r="G148" t="n">
+        <v>1</v>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>Kiểm tra D4</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:15Z</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:15Z</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:15Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000206</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Regression D6</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Test Item D6</t>
+        </is>
+      </c>
+      <c r="G149" t="n">
+        <v>1</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:16Z</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:16Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000207</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>other_user@company.com</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Other User</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Regression D7</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Test Item D7</t>
+        </is>
+      </c>
+      <c r="G150" t="n">
+        <v>1</v>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:16Z</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:16Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>REQ-20261009-000208</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Regression D8 Overdue</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Test Item D8</t>
+        </is>
+      </c>
+      <c r="G151" t="n">
+        <v>1</v>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:17Z</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:17Z</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:42:17Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(agent): implement low-stock inventory report capability (low_stock_inventory)
</commit_message>
<xml_diff>
--- a/backend/data/equipment_agent.xlsx
+++ b/backend/data/equipment_agent.xlsx
@@ -4518,7 +4518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U151"/>
+  <dimension ref="A1:U156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16275,6 +16275,401 @@
       <c r="U151" t="inlineStr">
         <is>
           <t>2026-10-09T13:42:17Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000209</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G152" t="n">
+        <v>1</v>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:30Z</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000210</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Regression D4</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Test Item D4</t>
+        </is>
+      </c>
+      <c r="G153" t="n">
+        <v>1</v>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Kiểm tra D4</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:32Z</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:32Z</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000211</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Regression D6</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Test Item D6</t>
+        </is>
+      </c>
+      <c r="G154" t="n">
+        <v>1</v>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:33Z</t>
+        </is>
+      </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:33Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000212</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>other_user@company.com</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Other User</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Regression D7</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Test Item D7</t>
+        </is>
+      </c>
+      <c r="G155" t="n">
+        <v>1</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:34Z</t>
+        </is>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:34Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000213</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Regression D8 Overdue</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Test Item D8</t>
+        </is>
+      </c>
+      <c r="G156" t="n">
+        <v>1</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:35Z</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:34Z</t>
+        </is>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>2026-10-10T04:42:35Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(format): escape pipe and special characters in Markdown table cells
</commit_message>
<xml_diff>
--- a/backend/data/equipment_agent.xlsx
+++ b/backend/data/equipment_agent.xlsx
@@ -4518,7 +4518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U156"/>
+  <dimension ref="A1:U161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5904,7 +5904,17 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Borrowed</t>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Nguyên trạng như khi nhận</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:22:56Z</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -5914,7 +5924,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>2025-09-21T09:00:00Z</t>
+          <t>2026-10-10T12:22:56Z</t>
         </is>
       </c>
     </row>
@@ -16670,6 +16680,401 @@
       <c r="U156" t="inlineStr">
         <is>
           <t>2026-10-10T04:42:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000214</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Test Project</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G157" t="n">
+        <v>1</v>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Testing regression C4</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:07Z</t>
+        </is>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:07Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000215</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Regression D4</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Test Item D4</t>
+        </is>
+      </c>
+      <c r="G158" t="n">
+        <v>1</v>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>Kiểm tra D4</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:07Z</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000216</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Regression D6</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Test Item D6</t>
+        </is>
+      </c>
+      <c r="G159" t="n">
+        <v>1</v>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000217</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>other_user@company.com</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Other User</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Regression D7</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Test Item D7</t>
+        </is>
+      </c>
+      <c r="G160" t="n">
+        <v>1</v>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>REQ-20261010-000218</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Nam Pham</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Regression D8 Overdue</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>TU1-003</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Test Item D8</t>
+        </is>
+      </c>
+      <c r="G161" t="n">
+        <v>1</v>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Regression test</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Test reason</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
+        </is>
+      </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:41:08Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(agent): resolve equipment context bleed and person overdue loan tracking
</commit_message>
<xml_diff>
--- a/backend/data/equipment_agent.xlsx
+++ b/backend/data/equipment_agent.xlsx
@@ -4518,7 +4518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U37"/>
+  <dimension ref="A1:U41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7485,6 +7485,306 @@
       <c r="U37" t="inlineStr">
         <is>
           <t>2026-10-08T16:25:48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>REQ-20261012-000095</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>nampham.31231023820@st.ueh.edu.vn</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Minilab</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>5</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Test borrow</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Đánh giá ưu tiên tự động không thành công. Quản lý vui lòng xem xét.</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>2026-10-12T01:56:31Z</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>2026-10-12T01:56:43Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>REQ-20261012-000096</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>nampham.31231023820@st.ueh.edu.vn</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Minilab</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>5</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Minilab testing</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Đánh giá ưu tiên tự động không thành công. Quản lý vui lòng xem xét.</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:18:30Z</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:18:48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>REQ-20261012-000097</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Nam Phạm</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Alpha test</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>CSW-002</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>ECU ABS 10.3MP</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Test flash software</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Đánh giá ưu tiên tự động không thành công. Quản lý vui lòng xem xét.</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:31:45Z</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:32:02Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>REQ-20261012-000098</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>phamngochainam25@gmail.com</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nam Phạm</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Alpha test</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TU1-001</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Conn header SMD 24pos 3mm female</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Đánh giá ưu tiên tự động không thành công. Quản lý vui lòng xem xét.</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>2026-10-12T20:01:00Z</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>2026-10-12T20:01:03Z</t>
         </is>
       </c>
     </row>
@@ -7499,7 +7799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34.109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7770,6 +8070,28 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>khiembao@gmail.com</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Khiembao</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MANAGER</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(approval): resolve partial return split and preserve manager rejection reason
</commit_message>
<xml_diff>
--- a/backend/data/equipment_agent.xlsx
+++ b/backend/data/equipment_agent.xlsx
@@ -4518,7 +4518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4627,6 +4627,11 @@
           <t>UpdatedAt</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>RejectionReason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4714,7 +4719,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-10-07T16:44:28Z</t>
+          <t>2026-10-14T20:28:03Z</t>
         </is>
       </c>
     </row>
@@ -7785,6 +7790,81 @@
       <c r="U41" t="inlineStr">
         <is>
           <t>2026-10-12T20:01:03Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>REQ-20261014-000099</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>dev@example.com</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Proj</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TU1-002</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Conn header R/A 10pos 4.2mm</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-11-25</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Chờ quản lý xem xét</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>2026-10-14T20:27:32Z</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>2026-10-14T20:27:32Z</t>
         </is>
       </c>
     </row>

</xml_diff>